<commit_message>
Spalten Land, Region und Website ergaenzt
Land und Region beziehen sich auf die adressierte Gesellschaft, nicht auf den
Konzernsitz - vier der zehn Haeuser sind US-Konzerne, angesprochen wird aber
jeweils die europaeische Einheit. Website ist in der Excel als klickbarer
Hyperlink hinterlegt und zeigt, wo vorhanden, auf die deutsche Praesenz.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015H8odxAEQBbyd5de8uHVVB
</commit_message>
<xml_diff>
--- a/Contact_Log_Consulting_Partner_DACH.xlsx
+++ b/Contact_Log_Consulting_Partner_DACH.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Contact Log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Contact Log'!$A$1:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Contact Log'!$A$1:$L$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,12 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -102,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -113,14 +119,17 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -486,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -498,6 +507,9 @@
     <col width="62" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -546,6 +558,21 @@
           <t>Adresse</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Land</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="50" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -589,6 +616,21 @@
           <t>Alvarez &amp; Marsal Deutschland GmbH, Sonnenstraße 20, 80331 München</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>https://www.germany-alvarezandmarsal.com</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="50" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -612,12 +654,12 @@
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>christian.saeuberlich@fti-andersch.com</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Firmenschema (zwei Belege: leoni.juschkat@ und ellina.hanxleden@fti-andersch.com; Umlaut-Schreibweise gestützt durch Seiten-URL .../management/christian-saeuberlich/) - Rückfall: info@fti-andersch.com</t>
         </is>
@@ -630,6 +672,21 @@
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>FTI-Andersch AG, Taunusanlage 9-10, 60329 Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.fti-andersch.com</t>
         </is>
       </c>
     </row>
@@ -655,12 +712,12 @@
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>geoff.rowley@frpadvisory.com</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>BESTÄTIGT - https://www.frpadvisory.com/about-us/our-people/geoff-rowley/</t>
         </is>
@@ -673,6 +730,21 @@
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>FRP Advisory Group plc, 110 Cannon Street, London EC4N 6EU, United Kingdom</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Vereinigtes Königreich</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>https://www.frpadvisory.com</t>
         </is>
       </c>
     </row>
@@ -716,6 +788,21 @@
       <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Investec Advisory GmbH &amp; Co. KG, Sonnenberger Straße 16, 65193 Wiesbaden</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>https://capitalmind.com</t>
         </is>
       </c>
     </row>
@@ -757,6 +844,21 @@
           <t>Piper Sandler Ltd., 2 Gresham Street, 6th Floor, London, United Kingdom</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Vereinigtes Königreich</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pipersandler.com</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="50" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -780,12 +882,12 @@
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>christian.stippler@stifel.com</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>BESTÄTIGT - https://stifelinstitutional.com/meet/christian-stippler/ (Adresse, Telefon und v-Card auf der Profilseite)</t>
         </is>
@@ -798,6 +900,21 @@
       <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Stifel Europe Advisory GmbH, Luginsland 1, 60313 Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.stifel.com</t>
         </is>
       </c>
     </row>
@@ -843,6 +960,21 @@
           <t>Forvis Mazars GmbH &amp; Co. KG, Domstraße 15, 20095 Hamburg</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.forvismazars.com/de/de</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="50" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -866,12 +998,12 @@
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>fabian.brandt@oliverwyman.com</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Firmenschema (drei Belege auf oliverwyman.de: felix.wilker@, davina.lermer-spitzweg@, aleksandar.nikolov@oliverwyman.com)</t>
         </is>
@@ -884,6 +1016,21 @@
       <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Oliver Wyman GmbH, Müllerstraße 3, 80469 München</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oliverwyman.de</t>
         </is>
       </c>
     </row>
@@ -909,12 +1056,12 @@
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>stefan.schaible@rolandberger.com</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Firmenschema (drei Belege im offiziellen Newsroom: silvia.zoesch@, julia.frank@, philipp.topitsch@rolandberger.com)</t>
         </is>
@@ -927,6 +1074,21 @@
       <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Roland Berger GmbH, Sederanger 1, 80538 München</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.rolandberger.com</t>
         </is>
       </c>
     </row>
@@ -948,12 +1110,12 @@
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>jens.nawrath@ankura.com</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Firmenschema, nur EIN Beleg (robin.boesen@ankura.com aus der offiziellen Pressemitteilung vom 14.08.2025) - vor Versand verifizieren</t>
         </is>
@@ -968,89 +1130,116 @@
           <t>Ankura Consulting Group, Taunusanlage 21, 60325 Frankfurt am Main</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>https://ankura.com</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Legende Spalte "Herkunft Email" (Farbe in Spalte Email/Herkunft)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>GRUEN  "BESTAETIGT" + URL = Adresse steht so auf der genannten offiziellen Unternehmensseite. Direkt verwendbar.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>GELB   "Firmenschema" = aus dem belegten Muster desselben Unternehmens gebildet, Mailbox nicht verifiziert. Anzahl der Belege ist jeweils genannt.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>GELB   "Allgemeiner offizieller Kontakt" = Funktionsadresse, weil kein persoenliches Postfach veroeffentlicht ist. Anschreiben mit Weiterleitungsbitte.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>ROT    "SCHWACH BELEGT" / "WIDERSPRUCH" / "WARNUNG" = Beleglage unzureichend oder Quellen widersprechen sich. Vor Versand zwingend pruefen.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr"/>
+      <c r="A18" s="8" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Weitere Hinweise</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Adresse = Sitz der adressierten Gesellschaft bzw. des adressierten Bueros. Abweichende Arbeitsorte: Dr. Regierer sitzt in Berlin (Alt-Moabit 2, 10557 Berlin), S. Schaible in Frankfurt (OpernTurm, Bockenheimer Landstr. 2-8, 60306 Frankfurt).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Alvarez &amp; Marsal: A&amp;M Deutschland wird von einem Trio gefuehrt - Juergen Zapf, Patrick Siebert, Bob Rajan. Deutsche Zentrale ist Muenchen, nicht Frankfurt. Einzige bestaetigte Direktadresse im deutschen Team: jstohner@alvarezandmarsal.com (Johann Stohner, Head of Restructuring Germany, Muenchen, Mobil +49 170 921 3836) - als Alternative mit gesicherter Adresse.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Stifel: DACH-Advisory-Fuehrung im Wechsel (J. Lucas ausgeschieden 11/2024, T. Klack seit 12/2025 nicht mehr Geschaeftsfuehrer). Stippler ist als MD Frankfurt und eingetragener Geschaeftsfuehrer belegt.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>FRP und Piper Sandler haben keine deutsche Partnerebene - Kontakt daher auf UK-Ebene.</t>
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>FRP und Piper Sandler haben keine deutsche Partnerebene - Kontakt daher auf UK-Ebene. Land und Region beziehen sich immer auf die adressierte Gesellschaft, nicht auf den Konzernsitz: Piper Sandler (Minneapolis), Stifel (St. Louis), Alvarez &amp; Marsal (New York) und Ankura (Washington D.C.) sind US-Haeuser, angesprochen wird aber jeweils die europaeische Einheit.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Telefonnummern sind Zentralen, sofern nicht als Durchwahl/Mobil ausgewiesen. Es wurden keine Test-Mails versendet.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I11"/>
+  <autoFilter ref="A1:L11"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>